<commit_message>
feat: initialize Oracle and SQL Server infrastructure including schema definitions, access controls, and replication jobs
</commit_message>
<xml_diff>
--- a/excel/MonthlyReport.xlsx
+++ b/excel/MonthlyReport.xlsx
@@ -413,10 +413,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
+    <row outlineLevel="0" r="1">
       <c r="A1" t="inlineStr">
         <is>
           <t>Miesiac</t>
@@ -428,7 +428,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row outlineLevel="0" r="2">
       <c r="A2" t="inlineStr">
         <is>
           <t>2026-05</t>
@@ -438,7 +438,7 @@
         <v>12000.5</v>
       </c>
     </row>
-    <row r="3">
+    <row outlineLevel="0" r="3">
       <c r="A3" t="inlineStr">
         <is>
           <t>2026-06</t>
@@ -446,6 +446,56 @@
       </c>
       <c r="B3" t="n">
         <v>15450.75</v>
+      </c>
+    </row>
+    <row outlineLevel="0" r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B4" s="0">
+        <v>11500</v>
+      </c>
+    </row>
+    <row outlineLevel="0" r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B5" s="0">
+        <v>9800.2</v>
+      </c>
+    </row>
+    <row outlineLevel="0" r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B6" s="0">
+        <v>10250.4</v>
+      </c>
+    </row>
+    <row outlineLevel="0" r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B7" s="0">
+        <v>14100.8</v>
+      </c>
+    </row>
+    <row outlineLevel="0" r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B8" s="0">
+        <v>13850.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>